<commit_message>
Cập nhật Video Demo và Hoàn thiện báo cáo
</commit_message>
<xml_diff>
--- a/Bang_tien_do_Smart_Agriculture_4_tuan.xlsx
+++ b/Bang_tien_do_Smart_Agriculture_4_tuan.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1e4638f2b6a0d9b9/Desktop/New folder (5)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nguye\Downloads\HK1_26-27\Uddd\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41589615-A388-4752-B9CA-B1CD017B23CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{808FFBCF-FDEB-4ECA-A753-FB2ABE58137E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -133,9 +133,6 @@
     <t>Tuấn &amp; Thắng &amp;Trí</t>
   </si>
   <si>
-    <t>Gồm cuốn Báo cáo, PPT thuyết trình, File tiến độ, Giphub</t>
-  </si>
-  <si>
     <t>Trình bày sản phầm cho thầy MRH3 xem, thầy nhận xét và đặt câu hỏi</t>
   </si>
   <si>
@@ -188,6 +185,9 @@
   </si>
   <si>
     <t>Toàn &amp; Tú</t>
+  </si>
+  <si>
+    <t>Gồm cuốn Báo cáo, PPT thuyết trình, File tiến độ, Github</t>
   </si>
 </sst>
 </file>
@@ -818,15 +818,6 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="46" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="47" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="48" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="49" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="50" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -838,9 +829,18 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="46" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1119,105 +1119,105 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BI60"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.59765625" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" customWidth="1"/>
     <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="61" width="3.59765625" customWidth="1"/>
+    <col min="7" max="61" width="3.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:61" ht="30.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="79" t="s">
+    <row r="1" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="79" t="s">
+      <c r="B1" s="76" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="79" t="s">
+      <c r="C1" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="79" t="s">
+      <c r="D1" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="79" t="s">
+      <c r="E1" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="79" t="s">
+      <c r="F1" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="71" t="s">
+      <c r="G1" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="71"/>
-      <c r="M1" s="71"/>
-      <c r="N1" s="71"/>
-      <c r="O1" s="72" t="s">
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="79" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="72"/>
-      <c r="Q1" s="72"/>
-      <c r="R1" s="72"/>
-      <c r="S1" s="72"/>
-      <c r="T1" s="72"/>
-      <c r="U1" s="72"/>
-      <c r="V1" s="72"/>
-      <c r="W1" s="72"/>
-      <c r="X1" s="72"/>
-      <c r="Y1" s="72"/>
-      <c r="Z1" s="72"/>
-      <c r="AA1" s="72"/>
-      <c r="AB1" s="72"/>
-      <c r="AC1" s="72"/>
-      <c r="AD1" s="72"/>
-      <c r="AE1" s="72"/>
-      <c r="AF1" s="72"/>
-      <c r="AG1" s="72"/>
-      <c r="AH1" s="72"/>
-      <c r="AI1" s="72"/>
-      <c r="AJ1" s="72"/>
-      <c r="AK1" s="72"/>
-      <c r="AL1" s="72"/>
-      <c r="AM1" s="72"/>
-      <c r="AN1" s="72"/>
-      <c r="AO1" s="72"/>
-      <c r="AP1" s="72"/>
-      <c r="AQ1" s="72"/>
-      <c r="AR1" s="72"/>
-      <c r="AS1" s="73" t="s">
+      <c r="P1" s="79"/>
+      <c r="Q1" s="79"/>
+      <c r="R1" s="79"/>
+      <c r="S1" s="79"/>
+      <c r="T1" s="79"/>
+      <c r="U1" s="79"/>
+      <c r="V1" s="79"/>
+      <c r="W1" s="79"/>
+      <c r="X1" s="79"/>
+      <c r="Y1" s="79"/>
+      <c r="Z1" s="79"/>
+      <c r="AA1" s="79"/>
+      <c r="AB1" s="79"/>
+      <c r="AC1" s="79"/>
+      <c r="AD1" s="79"/>
+      <c r="AE1" s="79"/>
+      <c r="AF1" s="79"/>
+      <c r="AG1" s="79"/>
+      <c r="AH1" s="79"/>
+      <c r="AI1" s="79"/>
+      <c r="AJ1" s="79"/>
+      <c r="AK1" s="79"/>
+      <c r="AL1" s="79"/>
+      <c r="AM1" s="79"/>
+      <c r="AN1" s="79"/>
+      <c r="AO1" s="79"/>
+      <c r="AP1" s="79"/>
+      <c r="AQ1" s="79"/>
+      <c r="AR1" s="79"/>
+      <c r="AS1" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="AT1" s="73"/>
-      <c r="AU1" s="73"/>
-      <c r="AV1" s="73"/>
-      <c r="AW1" s="73"/>
-      <c r="AX1" s="73"/>
-      <c r="AY1" s="73"/>
-      <c r="AZ1" s="73"/>
-      <c r="BA1" s="73"/>
-      <c r="BB1" s="73"/>
-      <c r="BC1" s="73"/>
-      <c r="BD1" s="73"/>
-      <c r="BE1" s="73"/>
-      <c r="BF1" s="73"/>
-      <c r="BG1" s="73"/>
-      <c r="BH1" s="73"/>
-      <c r="BI1" s="73"/>
-    </row>
-    <row r="2" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="80"/>
-      <c r="B2" s="80"/>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
+      <c r="AT1" s="80"/>
+      <c r="AU1" s="80"/>
+      <c r="AV1" s="80"/>
+      <c r="AW1" s="80"/>
+      <c r="AX1" s="80"/>
+      <c r="AY1" s="80"/>
+      <c r="AZ1" s="80"/>
+      <c r="BA1" s="80"/>
+      <c r="BB1" s="80"/>
+      <c r="BC1" s="80"/>
+      <c r="BD1" s="80"/>
+      <c r="BE1" s="80"/>
+      <c r="BF1" s="80"/>
+      <c r="BG1" s="80"/>
+      <c r="BH1" s="80"/>
+      <c r="BI1" s="80"/>
+    </row>
+    <row r="2" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="77"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
       <c r="G2" s="28">
         <v>24</v>
       </c>
@@ -1384,7 +1384,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>28</v>
       </c>
@@ -1459,7 +1459,7 @@
       <c r="BH3" s="21"/>
       <c r="BI3" s="21"/>
     </row>
-    <row r="4" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
@@ -1534,12 +1534,12 @@
       <c r="BH4" s="21"/>
       <c r="BI4" s="21"/>
     </row>
-    <row r="5" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
@@ -1609,7 +1609,7 @@
       <c r="BH5" s="21"/>
       <c r="BI5" s="21"/>
     </row>
-    <row r="6" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>28</v>
       </c>
@@ -1684,7 +1684,7 @@
       <c r="BH6" s="21"/>
       <c r="BI6" s="21"/>
     </row>
-    <row r="7" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>29</v>
       </c>
@@ -1759,12 +1759,12 @@
       <c r="BH7" s="21"/>
       <c r="BI7" s="21"/>
     </row>
-    <row r="8" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>10</v>
@@ -1834,7 +1834,7 @@
       <c r="BH8" s="21"/>
       <c r="BI8" s="21"/>
     </row>
-    <row r="9" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>29</v>
       </c>
@@ -1909,12 +1909,12 @@
       <c r="BH9" s="21"/>
       <c r="BI9" s="21"/>
     </row>
-    <row r="10" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>12</v>
@@ -1984,12 +1984,12 @@
       <c r="BH10" s="23"/>
       <c r="BI10" s="21"/>
     </row>
-    <row r="11" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>13</v>
@@ -2059,12 +2059,12 @@
       <c r="BH11" s="21"/>
       <c r="BI11" s="21"/>
     </row>
-    <row r="12" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>14</v>
@@ -2134,12 +2134,12 @@
       <c r="BH12" s="21"/>
       <c r="BI12" s="21"/>
     </row>
-    <row r="13" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>15</v>
@@ -2209,12 +2209,12 @@
       <c r="BH13" s="24"/>
       <c r="BI13" s="24"/>
     </row>
-    <row r="14" spans="1:61" ht="32" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:61" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>16</v>
@@ -2284,15 +2284,15 @@
       <c r="BH14" s="21"/>
       <c r="BI14" s="21"/>
     </row>
-    <row r="15" spans="1:61" ht="31.8" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:61" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D15" s="67">
         <v>46281</v>
@@ -2359,15 +2359,15 @@
       <c r="BH15" s="21"/>
       <c r="BI15" s="21"/>
     </row>
-    <row r="16" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D16" s="67">
         <v>46283</v>
@@ -2434,12 +2434,12 @@
       <c r="BH16" s="21"/>
       <c r="BI16" s="21"/>
     </row>
-    <row r="17" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="18" t="s">
         <v>33</v>
       </c>
       <c r="B17" s="34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>18</v>
@@ -2509,12 +2509,12 @@
       <c r="BH17" s="21"/>
       <c r="BI17" s="21"/>
     </row>
-    <row r="18" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="18" t="s">
         <v>33</v>
       </c>
       <c r="B18" s="34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>19</v>
@@ -2584,15 +2584,15 @@
       <c r="BH18" s="21"/>
       <c r="BI18" s="21"/>
     </row>
-    <row r="19" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="64" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="65" t="s">
+      <c r="C19" s="7" t="s">
         <v>45</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>46</v>
       </c>
       <c r="D19" s="69" t="s">
         <v>22</v>
@@ -2601,7 +2601,7 @@
         <v>7</v>
       </c>
       <c r="F19" s="69" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G19" s="21"/>
       <c r="H19" s="21"/>
@@ -2631,13 +2631,13 @@
       <c r="AF19" s="22"/>
       <c r="AG19" s="22"/>
       <c r="AH19" s="21"/>
-      <c r="AI19" s="74"/>
-      <c r="AJ19" s="74"/>
-      <c r="AK19" s="74"/>
-      <c r="AL19" s="74"/>
-      <c r="AM19" s="75"/>
-      <c r="AN19" s="76"/>
-      <c r="AO19" s="76"/>
+      <c r="AI19" s="71"/>
+      <c r="AJ19" s="71"/>
+      <c r="AK19" s="71"/>
+      <c r="AL19" s="71"/>
+      <c r="AM19" s="72"/>
+      <c r="AN19" s="73"/>
+      <c r="AO19" s="73"/>
       <c r="AP19" s="21"/>
       <c r="AQ19" s="21"/>
       <c r="AR19" s="21"/>
@@ -2659,24 +2659,24 @@
       <c r="BH19" s="21"/>
       <c r="BI19" s="21"/>
     </row>
-    <row r="20" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B20" s="35" t="s">
         <v>35</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="D20" s="69" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E20" s="70">
         <v>8</v>
       </c>
       <c r="F20" s="69" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
@@ -2715,7 +2715,7 @@
       <c r="AO20" s="21"/>
       <c r="AP20" s="66"/>
       <c r="AQ20" s="66"/>
-      <c r="AR20" s="77"/>
+      <c r="AR20" s="74"/>
       <c r="AS20" s="21"/>
       <c r="AT20" s="22"/>
       <c r="AU20" s="22"/>
@@ -2734,24 +2734,24 @@
       <c r="BH20" s="21"/>
       <c r="BI20" s="21"/>
     </row>
-    <row r="21" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B21" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D21" s="69" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E21" s="70">
         <v>1</v>
       </c>
       <c r="F21" s="69" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
@@ -2790,7 +2790,7 @@
       <c r="AO21" s="21"/>
       <c r="AP21" s="21"/>
       <c r="AQ21" s="21"/>
-      <c r="AR21" s="78"/>
+      <c r="AR21" s="75"/>
       <c r="AS21" s="27"/>
       <c r="AT21" s="27"/>
       <c r="AU21" s="22"/>
@@ -2809,7 +2809,7 @@
       <c r="BH21" s="21"/>
       <c r="BI21" s="21"/>
     </row>
-    <row r="22" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="32"/>
       <c r="B22" s="36"/>
       <c r="C22" s="7"/>
@@ -2872,7 +2872,7 @@
       <c r="BH22" s="21"/>
       <c r="BI22" s="21"/>
     </row>
-    <row r="23" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="32"/>
       <c r="B23" s="36"/>
       <c r="C23" s="7"/>
@@ -2935,7 +2935,7 @@
       <c r="BH23" s="12"/>
       <c r="BI23" s="12"/>
     </row>
-    <row r="24" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="32"/>
       <c r="B24" s="36"/>
       <c r="C24" s="7"/>
@@ -2998,7 +2998,7 @@
       <c r="BH24" s="12"/>
       <c r="BI24" s="12"/>
     </row>
-    <row r="25" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="32"/>
       <c r="B25" s="36"/>
       <c r="C25" s="7"/>
@@ -3061,7 +3061,7 @@
       <c r="BH25" s="12"/>
       <c r="BI25" s="12"/>
     </row>
-    <row r="26" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="32"/>
       <c r="B26" s="33"/>
       <c r="C26" s="7"/>
@@ -3124,7 +3124,7 @@
       <c r="BH26" s="12"/>
       <c r="BI26" s="12"/>
     </row>
-    <row r="27" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="32"/>
       <c r="B27" s="33"/>
       <c r="C27" s="7"/>
@@ -3144,7 +3144,7 @@
       <c r="Q27" s="12"/>
       <c r="R27" s="12"/>
     </row>
-    <row r="28" spans="1:61" ht="30.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:61" ht="30.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="32"/>
       <c r="B28" s="33"/>
       <c r="C28" s="7"/>
@@ -3164,7 +3164,7 @@
       <c r="Q28" s="12"/>
       <c r="R28" s="12"/>
     </row>
-    <row r="29" spans="1:61" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A29" s="6"/>
       <c r="B29" s="17"/>
       <c r="C29" s="7"/>
@@ -3184,7 +3184,7 @@
       <c r="Q29" s="12"/>
       <c r="R29" s="12"/>
     </row>
-    <row r="30" spans="1:61" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
       <c r="B30" s="17"/>
       <c r="C30" s="7"/>
@@ -3204,7 +3204,7 @@
       <c r="Q30" s="12"/>
       <c r="R30" s="12"/>
     </row>
-    <row r="31" spans="1:61" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
       <c r="B31" s="17"/>
       <c r="C31" s="7"/>
@@ -3224,7 +3224,7 @@
       <c r="Q31" s="12"/>
       <c r="R31" s="12"/>
     </row>
-    <row r="32" spans="1:61" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
       <c r="B32" s="17"/>
       <c r="C32" s="7"/>
@@ -3244,7 +3244,7 @@
       <c r="Q32" s="12"/>
       <c r="R32" s="12"/>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
       <c r="B33" s="17"/>
       <c r="C33" s="7"/>
@@ -3264,7 +3264,7 @@
       <c r="Q33" s="12"/>
       <c r="R33" s="12"/>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A34" s="6"/>
       <c r="B34" s="17"/>
       <c r="C34" s="7"/>
@@ -3284,7 +3284,7 @@
       <c r="Q34" s="12"/>
       <c r="R34" s="12"/>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A35" s="6"/>
       <c r="B35" s="17"/>
       <c r="C35" s="7"/>
@@ -3304,7 +3304,7 @@
       <c r="Q35" s="12"/>
       <c r="R35" s="12"/>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A36" s="6"/>
       <c r="B36" s="17"/>
       <c r="C36" s="7"/>
@@ -3324,7 +3324,7 @@
       <c r="Q36" s="12"/>
       <c r="R36" s="12"/>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A37" s="6"/>
       <c r="B37" s="17"/>
       <c r="C37" s="7"/>
@@ -3344,7 +3344,7 @@
       <c r="Q37" s="12"/>
       <c r="R37" s="12"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A38" s="6"/>
       <c r="B38" s="17"/>
       <c r="C38" s="7"/>
@@ -3364,7 +3364,7 @@
       <c r="Q38" s="12"/>
       <c r="R38" s="12"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A39" s="6"/>
       <c r="B39" s="17"/>
       <c r="C39" s="7"/>
@@ -3384,7 +3384,7 @@
       <c r="Q39" s="12"/>
       <c r="R39" s="12"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A40" s="6"/>
       <c r="B40" s="17"/>
       <c r="C40" s="7"/>
@@ -3404,7 +3404,7 @@
       <c r="Q40" s="12"/>
       <c r="R40" s="12"/>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A41" s="6"/>
       <c r="B41" s="17"/>
       <c r="C41" s="7"/>
@@ -3424,7 +3424,7 @@
       <c r="Q41" s="12"/>
       <c r="R41" s="12"/>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A42" s="6"/>
       <c r="B42" s="17"/>
       <c r="C42" s="7"/>
@@ -3444,7 +3444,7 @@
       <c r="Q42" s="12"/>
       <c r="R42" s="12"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A43" s="6"/>
       <c r="B43" s="17"/>
       <c r="C43" s="7"/>
@@ -3464,7 +3464,7 @@
       <c r="Q43" s="12"/>
       <c r="R43" s="12"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A44" s="6"/>
       <c r="B44" s="17"/>
       <c r="C44" s="7"/>
@@ -3484,7 +3484,7 @@
       <c r="Q44" s="12"/>
       <c r="R44" s="12"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A45" s="6"/>
       <c r="B45" s="17"/>
       <c r="C45" s="7"/>
@@ -3504,7 +3504,7 @@
       <c r="Q45" s="12"/>
       <c r="R45" s="12"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A46" s="6"/>
       <c r="B46" s="17"/>
       <c r="C46" s="7"/>
@@ -3524,7 +3524,7 @@
       <c r="Q46" s="12"/>
       <c r="R46" s="12"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A47" s="6"/>
       <c r="B47" s="17"/>
       <c r="C47" s="7"/>
@@ -3544,7 +3544,7 @@
       <c r="Q47" s="12"/>
       <c r="R47" s="12"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A48" s="6"/>
       <c r="B48" s="17"/>
       <c r="C48" s="7"/>
@@ -3564,7 +3564,7 @@
       <c r="Q48" s="12"/>
       <c r="R48" s="12"/>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A49" s="6"/>
       <c r="B49" s="17"/>
       <c r="C49" s="7"/>
@@ -3584,7 +3584,7 @@
       <c r="Q49" s="12"/>
       <c r="R49" s="12"/>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A50" s="6"/>
       <c r="B50" s="17"/>
       <c r="C50" s="7"/>
@@ -3604,7 +3604,7 @@
       <c r="Q50" s="12"/>
       <c r="R50" s="12"/>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A51" s="6"/>
       <c r="B51" s="17"/>
       <c r="C51" s="7"/>
@@ -3624,7 +3624,7 @@
       <c r="Q51" s="12"/>
       <c r="R51" s="12"/>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A52" s="6"/>
       <c r="B52" s="17"/>
       <c r="C52" s="7"/>
@@ -3644,7 +3644,7 @@
       <c r="Q52" s="12"/>
       <c r="R52" s="12"/>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A53" s="6"/>
       <c r="B53" s="17"/>
       <c r="C53" s="7"/>
@@ -3664,7 +3664,7 @@
       <c r="Q53" s="12"/>
       <c r="R53" s="12"/>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A54" s="6"/>
       <c r="B54" s="17"/>
       <c r="C54" s="7"/>
@@ -3684,7 +3684,7 @@
       <c r="Q54" s="12"/>
       <c r="R54" s="12"/>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A55" s="6"/>
       <c r="B55" s="17"/>
       <c r="C55" s="7"/>
@@ -3704,7 +3704,7 @@
       <c r="Q55" s="12"/>
       <c r="R55" s="12"/>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A56" s="6"/>
       <c r="B56" s="17"/>
       <c r="C56" s="7"/>
@@ -3724,7 +3724,7 @@
       <c r="Q56" s="12"/>
       <c r="R56" s="12"/>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A57" s="6"/>
       <c r="B57" s="17"/>
       <c r="C57" s="7"/>
@@ -3744,7 +3744,7 @@
       <c r="Q57" s="12"/>
       <c r="R57" s="12"/>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A58" s="6"/>
       <c r="B58" s="17"/>
       <c r="C58" s="7"/>
@@ -3764,7 +3764,7 @@
       <c r="Q58" s="12"/>
       <c r="R58" s="12"/>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A59" s="6"/>
       <c r="B59" s="17"/>
       <c r="C59" s="7"/>
@@ -3784,7 +3784,7 @@
       <c r="Q59" s="12"/>
       <c r="R59" s="12"/>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A60" s="12"/>
       <c r="B60" s="12"/>
       <c r="C60" s="12"/>
@@ -3807,15 +3807,15 @@
   </sheetData>
   <autoFilter ref="A1:F15" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="9">
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:N1"/>
+    <mergeCell ref="O1:AR1"/>
+    <mergeCell ref="AS1:BI1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:N1"/>
-    <mergeCell ref="O1:AR1"/>
-    <mergeCell ref="AS1:BI1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>